<commit_message>
ADR 0005 v2 (checkpoint aprovado, ressalvas aplicadas); pergunta 20
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/medidas/comparacao-banco.xlsx
+++ b/docs/medidas/comparacao-banco.xlsx
@@ -551,11 +551,11 @@
         <v>4</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>50–59 ms vs ~91 ms; ambos sub-segundo (benchmark-banco-2026-10-10.md §4)</t>
+          <t>Timescale 50–59 ms vs MySQL 82–90 ms (buffer pool 2 GB); ambos sub-segundo (benchmark §4)</t>
         </is>
       </c>
     </row>
@@ -859,11 +859,11 @@
         <v>1.12</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1.24</v>
+        <v>1.38</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>EXPLAIN ANALYZE; Timescale com compr.: 1,12–1,19; MySQL particionado 1,24–1,71</t>
+          <t>EXPLAIN ANALYZE; Timescale com compr.: 1,12–1,19; MySQL particionado 1,24–1,71; MySQL c/ 2 GB: 1,38–1,68</t>
         </is>
       </c>
     </row>
@@ -882,11 +882,11 @@
         <v>58.7</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>90.59999999999999</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Timescale com compr. 58,7–59,2 (sem compr. 49,9–50,2); MySQL 90,6–116</t>
+          <t>Timescale com compr. 58,7–59,2 (sem compr. 49,9–50,2); MySQL 90,6–116; MySQL c/ buffer pool 128 MB: 90,6–116; c/ 2 GB: 82,6–90,4. PG shared_buffers 5,9 GB</t>
         </is>
       </c>
     </row>

</xml_diff>